<commit_message>
Some changes in framework
</commit_message>
<xml_diff>
--- a/src/test/resources/DataTest.xlsx
+++ b/src/test/resources/DataTest.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>NavItems</t>
   </si>
@@ -62,14 +62,17 @@
     <t>Please enter valid 10 digit mobile number.</t>
   </si>
   <si>
-    <t>.</t>
+    <t>Rest of India</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +89,12 @@
       <sz val="12"/>
       <color rgb="FF721C24"/>
       <name val="Source Sans Pro"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -129,13 +138,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,10 +450,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -499,6 +509,11 @@
     <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -526,7 +541,7 @@
     </row>
     <row r="2" spans="1:2" ht="15.75">
       <c r="A2" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>13</v>

</xml_diff>